<commit_message>
stage2: add skill and projectile property stores
</commit_message>
<xml_diff>
--- a/Excels/Excels/B-Battle_战斗表.xlsx
+++ b/Excels/Excels/B-Battle_战斗表.xlsx
@@ -3214,11 +3214,11 @@
       </c>
       <c r="G7" s="28" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Projectile</t>
         </is>
       </c>
       <c r="H7" s="28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I7" s="28" t="inlineStr">
         <is>
@@ -3264,11 +3264,11 @@
       </c>
       <c r="G8" s="28" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Projectile</t>
         </is>
       </c>
       <c r="H8" s="28" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I8" s="28" t="inlineStr">
         <is>
@@ -3314,11 +3314,11 @@
       </c>
       <c r="G9" s="28" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Projectile</t>
         </is>
       </c>
       <c r="H9" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I9" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
stage3: add modifier source rollback
</commit_message>
<xml_diff>
--- a/Excels/Excels/B-Battle_战斗表.xlsx
+++ b/Excels/Excels/B-Battle_战斗表.xlsx
@@ -953,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="7.7734375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9.1" customWidth="1" style="11" min="1" max="3"/>
@@ -1021,6 +1021,11 @@
           <t>endEffects</t>
         </is>
       </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>modifiers</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="12">
       <c r="A2" s="14" t="inlineStr">
@@ -1078,6 +1083,11 @@
           <t>(array#sep=|),Battle.EffectRef</t>
         </is>
       </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>(array#sep=|),Battle.BattleModifierRef</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="A3" s="15" t="inlineStr">
@@ -1135,6 +1145,11 @@
           <t>c</t>
         </is>
       </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="12">
       <c r="A4" s="16" t="inlineStr">
@@ -1190,6 +1205,11 @@
       <c r="K4" s="17" t="inlineStr">
         <is>
           <t>结束效果</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>????</t>
         </is>
       </c>
     </row>
@@ -1248,6 +1268,39 @@
       <c r="H6" s="18" t="inlineStr">
         <is>
           <t>104,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="11" t="n">
+        <v>7003</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>???????</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>99</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>Skill;1;Int,1;Null,0,0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
stage4: add trigger modifier runtime
</commit_message>
<xml_diff>
--- a/Excels/Excels/B-Battle_战斗表.xlsx
+++ b/Excels/Excels/B-Battle_战斗表.xlsx
@@ -2875,7 +2875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="12" min="1" max="1"/>
@@ -2923,32 +2923,37 @@
           <t>skillSelector</t>
         </is>
       </c>
-      <c r="G1" s="21" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>triggerEventType</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
         <is>
           <t>targetType</t>
         </is>
       </c>
-      <c r="H1" s="21" t="inlineStr">
+      <c r="I1" s="21" t="inlineStr">
         <is>
           <t>modifierType</t>
         </is>
       </c>
-      <c r="I1" s="21" t="inlineStr">
+      <c r="J1" s="21" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="J1" s="21" t="inlineStr">
+      <c r="K1" s="21" t="inlineStr">
         <is>
           <t>effect</t>
         </is>
       </c>
-      <c r="K1" s="21" t="inlineStr">
+      <c r="L1" s="21" t="inlineStr">
         <is>
           <t>maxStack</t>
         </is>
       </c>
-      <c r="L1" s="21" t="inlineStr">
+      <c r="M1" s="21" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
@@ -2985,32 +2990,37 @@
           <t>Battle.SkillSelector</t>
         </is>
       </c>
-      <c r="G2" s="23" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Battle.TriggerEventType</t>
+        </is>
+      </c>
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Battle.ModifierTargetType</t>
         </is>
       </c>
-      <c r="H2" s="23" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="I2" s="23" t="inlineStr">
+      <c r="J2" s="23" t="inlineStr">
         <is>
           <t>Battle.ModifierValue</t>
         </is>
       </c>
-      <c r="J2" s="23" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>Battle.EffectRef</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr">
+      <c r="L2" s="23" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="L2" s="23" t="inlineStr">
+      <c r="M2" s="23" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -3047,7 +3057,7 @@
           <t>c</t>
         </is>
       </c>
-      <c r="G3" s="25" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>c</t>
         </is>
@@ -3073,6 +3083,11 @@
         </is>
       </c>
       <c r="L3" s="25" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="M3" s="25" t="inlineStr">
         <is>
           <t>c</t>
         </is>
@@ -3109,32 +3124,37 @@
           <t>技能筛选</t>
         </is>
       </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>??????</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="inlineStr">
         <is>
           <t>目标类型</t>
         </is>
       </c>
-      <c r="H4" s="27" t="inlineStr">
+      <c r="I4" s="27" t="inlineStr">
         <is>
           <t>强化类型</t>
         </is>
       </c>
-      <c r="I4" s="27" t="inlineStr">
+      <c r="J4" s="27" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="K4" s="27" t="inlineStr">
         <is>
           <t>效果</t>
         </is>
       </c>
-      <c r="K4" s="27" t="inlineStr">
+      <c r="L4" s="27" t="inlineStr">
         <is>
           <t>最大层数</t>
         </is>
       </c>
-      <c r="L4" s="27" t="inlineStr">
+      <c r="M4" s="27" t="inlineStr">
         <is>
           <t>权重</t>
         </is>
@@ -3165,28 +3185,33 @@
           <t>0,</t>
         </is>
       </c>
-      <c r="G5" s="28" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="H5" s="28" t="n">
+      <c r="I5" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="28" t="inlineStr">
+      <c r="J5" s="28" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="J5" s="28" t="inlineStr">
+      <c r="K5" s="28" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="K5" s="28" t="n">
+      <c r="L5" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="L5" s="28" t="n">
+      <c r="M5" s="28" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3215,28 +3240,33 @@
           <t>0,</t>
         </is>
       </c>
-      <c r="G6" s="28" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="I6" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="28" t="inlineStr">
+      <c r="J6" s="28" t="inlineStr">
         <is>
           <t>RatioBp,2000</t>
         </is>
       </c>
-      <c r="J6" s="28" t="inlineStr">
+      <c r="K6" s="28" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="L6" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="28" t="n">
+      <c r="M6" s="28" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3265,28 +3295,33 @@
           <t>0,</t>
         </is>
       </c>
-      <c r="G7" s="28" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="H7" s="28" t="n">
+      <c r="I7" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="28" t="inlineStr">
+      <c r="J7" s="28" t="inlineStr">
         <is>
           <t>Int,6003</t>
         </is>
       </c>
-      <c r="J7" s="28" t="inlineStr">
+      <c r="K7" s="28" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="K7" s="28" t="n">
+      <c r="L7" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="28" t="n">
+      <c r="M7" s="28" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3315,28 +3350,33 @@
           <t>0,</t>
         </is>
       </c>
-      <c r="G8" s="28" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="I8" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="I8" s="28" t="inlineStr">
+      <c r="J8" s="28" t="inlineStr">
         <is>
           <t>Int,1200</t>
         </is>
       </c>
-      <c r="J8" s="28" t="inlineStr">
+      <c r="K8" s="28" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="L8" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="28" t="n">
+      <c r="M8" s="28" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3365,29 +3405,142 @@
           <t>0,</t>
         </is>
       </c>
-      <c r="G9" s="28" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="I9" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="28" t="inlineStr">
+      <c r="J9" s="28" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="J9" s="28" t="inlineStr">
+      <c r="K9" s="28" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="K9" s="28" t="n">
+      <c r="L9" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="28" t="n">
+      <c r="M9" s="28" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="11" t="n">
+        <v>9201</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>????????????????</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>OnSkillCast</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Int,1</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>Damage,3001,10000</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="n">
+        <v>9202</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>????????????????????</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0,2002</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OnProjectileHit</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Int,1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Damage,3001,10000</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stage5: expand roguelike enhancement pool
</commit_message>
<xml_diff>
--- a/Excels/Excels/B-Battle_战斗表.xlsx
+++ b/Excels/Excels/B-Battle_战斗表.xlsx
@@ -2875,7 +2875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="12" min="1" max="1"/>
@@ -2958,6 +2958,41 @@
           <t>weight</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>iconKey</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>rarity</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>conflictTags</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>requireEnhancementIds</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>excludeEnhancementIds</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>nextEnhancementIds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
@@ -3025,6 +3060,41 @@
           <t>int</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Battle.EnhancementRarity</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>(array#sep=|),string</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>(array#sep=|),string</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>(array#sep=|),int</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>(array#sep=|),int</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>(array#sep=|),int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -3092,6 +3162,41 @@
           <t>c</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
@@ -3157,6 +3262,41 @@
       <c r="M4" s="27" t="inlineStr">
         <is>
           <t>权重</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>??Key</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>????</t>
         </is>
       </c>
     </row>
@@ -3214,6 +3354,29 @@
       <c r="M5" s="28" t="n">
         <v>100</v>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>enhance_multi_arrow</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>9011</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="n"/>
@@ -3269,6 +3432,29 @@
       <c r="M6" s="28" t="n">
         <v>100</v>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>enhance_rapid_shot</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>9012</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="n"/>
@@ -3324,6 +3510,33 @@
       <c r="M7" s="28" t="n">
         <v>100</v>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>enhance_fireball_arrow</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>??|??|??</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>9013</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="n"/>
@@ -3379,6 +3592,29 @@
       <c r="M8" s="28" t="n">
         <v>100</v>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>enhance_blast_arrow</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>9014</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="n"/>
@@ -3434,6 +3670,29 @@
       <c r="M9" s="28" t="n">
         <v>100</v>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>enhance_pierce_arrow</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>9015</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="11" t="n">
@@ -3488,60 +3747,483 @@
       <c r="M10" s="11" t="n">
         <v>10</v>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>enhance_power_draw</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" t="n">
+      <c r="B11" s="11" t="n">
         <v>9202</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>????????????????????</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Hero,None,None,None,</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>0,2002</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>OnProjectileHit</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>Damage,3001,10000</t>
         </is>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="11" t="n">
         <v>10</v>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>enhance_chase_arrow</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>??|??|??</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" t="n">
+        <v>9011</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>??? II</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>??????????????</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Int,1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Null,0,0</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>60</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>enhance_multi_arrow_2</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>9001</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>9012</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>????????????20%?</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>RatioBp,2000</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Null,0,0</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>60</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>enhance_rapid_shot_2</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>9013</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>??????????????</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OnProjectileHit</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Int,1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Damage,3003,10000</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>50</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>enhance_fireball_arrow_2</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>??|??|??</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>9014</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>??? II</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>?????????????</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Projectile</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Int,600</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Null,0,0</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>60</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>enhance_blast_arrow_2</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>9015</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>??? II</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>????????????1????</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Projectile</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Int,1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Null,0,0</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>60</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>enhance_pierce_arrow_2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>??|??</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
modifier: add unit selector camp filter
</commit_message>
<xml_diff>
--- a/Excels/Excels/B-Battle_战斗表.xlsx
+++ b/Excels/Excels/B-Battle_战斗表.xlsx
@@ -2958,37 +2958,37 @@
           <t>weight</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>iconKey</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>rarity</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>conflictTags</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>requireEnhancementIds</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>excludeEnhancementIds</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="11" t="inlineStr">
         <is>
           <t>nextEnhancementIds</t>
         </is>
@@ -3060,37 +3060,37 @@
           <t>int</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>Battle.EnhancementRarity</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>(array#sep=|),string</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>(array#sep=|),string</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="11" t="inlineStr">
         <is>
           <t>(array#sep=|),int</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="11" t="inlineStr">
         <is>
           <t>(array#sep=|),int</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="11" t="inlineStr">
         <is>
           <t>(array#sep=|),int</t>
         </is>
@@ -3162,37 +3162,37 @@
           <t>c</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="N3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" s="11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>c</t>
         </is>
@@ -3264,37 +3264,37 @@
           <t>权重</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="11" t="inlineStr">
         <is>
           <t>??Key</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="11" t="inlineStr">
         <is>
           <t>??</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="11" t="inlineStr">
         <is>
           <t>??</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -3354,25 +3354,25 @@
       <c r="M5" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N5" s="11" t="inlineStr">
         <is>
           <t>enhance_multi_arrow</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="11" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
+      <c r="Q5" s="11" t="inlineStr"/>
+      <c r="R5" s="11" t="inlineStr"/>
+      <c r="S5" s="11" t="inlineStr"/>
+      <c r="T5" s="11" t="inlineStr">
         <is>
           <t>9011</t>
         </is>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F6" s="28" t="inlineStr">
@@ -3432,25 +3432,25 @@
       <c r="M6" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>enhance_rapid_shot</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="11" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr">
+      <c r="Q6" s="11" t="inlineStr"/>
+      <c r="R6" s="11" t="inlineStr"/>
+      <c r="S6" s="11" t="inlineStr"/>
+      <c r="T6" s="11" t="inlineStr">
         <is>
           <t>9012</t>
         </is>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -3510,29 +3510,29 @@
       <c r="M7" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>enhance_fireball_arrow</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="11" t="inlineStr">
         <is>
           <t>??|??|??</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q7" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
+      <c r="R7" s="11" t="inlineStr"/>
+      <c r="S7" s="11" t="inlineStr"/>
+      <c r="T7" s="11" t="inlineStr">
         <is>
           <t>9013</t>
         </is>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="E8" s="28" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F8" s="28" t="inlineStr">
@@ -3592,25 +3592,25 @@
       <c r="M8" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N8" s="11" t="inlineStr">
         <is>
           <t>enhance_blast_arrow</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
+      <c r="Q8" s="11" t="inlineStr"/>
+      <c r="R8" s="11" t="inlineStr"/>
+      <c r="S8" s="11" t="inlineStr"/>
+      <c r="T8" s="11" t="inlineStr">
         <is>
           <t>9014</t>
         </is>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -3670,25 +3670,25 @@
       <c r="M9" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N9" s="11" t="inlineStr">
         <is>
           <t>enhance_pierce_arrow</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="11" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr">
+      <c r="Q9" s="11" t="inlineStr"/>
+      <c r="R9" s="11" t="inlineStr"/>
+      <c r="S9" s="11" t="inlineStr"/>
+      <c r="T9" s="11" t="inlineStr">
         <is>
           <t>9015</t>
         </is>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -3747,25 +3747,25 @@
       <c r="M10" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N10" s="11" t="inlineStr">
         <is>
           <t>enhance_power_draw</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
+      <c r="Q10" s="11" t="inlineStr"/>
+      <c r="R10" s="11" t="inlineStr"/>
+      <c r="S10" s="11" t="inlineStr"/>
+      <c r="T10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="B11" s="11" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Hero,None,None,None,</t>
+          <t>Hero,None,None,None,Player,</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -3820,410 +3820,410 @@
       <c r="M11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>enhance_chase_arrow</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" s="11" t="inlineStr">
         <is>
           <t>??|??|??</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
+      <c r="Q11" s="11" t="inlineStr"/>
+      <c r="R11" s="11" t="inlineStr"/>
+      <c r="S11" s="11" t="inlineStr"/>
+      <c r="T11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" t="n">
+      <c r="B12" s="11" t="n">
         <v>9011</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>??? II</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>??????????????</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Hero,None,None,None,</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,Player,</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>0,</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>enhance_multi_arrow_2</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
+      <c r="Q12" s="11" t="inlineStr"/>
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>9001</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="S12" s="11" t="inlineStr"/>
+      <c r="T12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" t="n">
+      <c r="B13" s="11" t="n">
         <v>9012</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>????????????20%?</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Hero,None,None,None,</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,Player,</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>0,</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>RatioBp,2000</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>enhance_rapid_shot_2</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
+      <c r="Q13" s="11" t="inlineStr"/>
+      <c r="R13" s="11" t="inlineStr">
         <is>
           <t>9002</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="B14" t="n">
+      <c r="B14" s="11" t="n">
         <v>9013</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>????</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>??????????????</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Hero,None,None,None,</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,Player,</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>0,</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>OnProjectileHit</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>Damage,3003,10000</t>
         </is>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N14" s="11" t="inlineStr">
         <is>
           <t>enhance_fireball_arrow_2</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="11" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P14" s="11" t="inlineStr">
         <is>
           <t>??|??|??</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
+      <c r="Q14" s="11" t="inlineStr"/>
+      <c r="R14" s="11" t="inlineStr">
         <is>
           <t>9003</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" t="n">
+      <c r="B15" s="11" t="n">
         <v>9014</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>??? II</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>?????????????</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Hero,None,None,None,</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,Player,</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>0,</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>Int,600</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>enhance_blast_arrow_2</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
+      <c r="Q15" s="11" t="inlineStr"/>
+      <c r="R15" s="11" t="inlineStr">
         <is>
           <t>9004</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" t="n">
+      <c r="B16" s="11" t="n">
         <v>9015</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>??? II</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>????????????1????</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Hero,None,None,None,</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Hero,None,None,None,Player,</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>0,</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr">
         <is>
           <t>Int,1</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>Null,0,0</t>
         </is>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N16" s="11" t="inlineStr">
         <is>
           <t>enhance_pierce_arrow_2</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="11" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" s="11" t="inlineStr">
         <is>
           <t>??|??</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
+      <c r="Q16" s="11" t="inlineStr"/>
+      <c r="R16" s="11" t="inlineStr">
         <is>
           <t>9005</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>